<commit_message>
modified structure for generating polio results. Added test mmr results
</commit_message>
<xml_diff>
--- a/src/Data/country_data.xlsx
+++ b/src/Data/country_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rafaelleon/polio-risk-assessment/src/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47E558B-1E8D-D14B-8EF5-9C034A137125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FDF8FF7-956B-A447-8438-8DF4702EF272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38980" yWindow="3360" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{7CFA64C4-648F-B840-901A-EC2D94882293}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" xr2:uid="{7CFA64C4-648F-B840-901A-EC2D94882293}"/>
   </bookViews>
   <sheets>
     <sheet name="1-General" sheetId="1" r:id="rId1"/>
@@ -350,9 +350,6 @@
     <t>Esquema de vacunación contra la polio</t>
   </si>
   <si>
-    <t>SPA</t>
-  </si>
-  <si>
     <t>Belize</t>
   </si>
   <si>
@@ -396,6 +393,9 @@
   </si>
   <si>
     <t>TOLEDO</t>
+  </si>
+  <si>
+    <t>ENG</t>
   </si>
 </sst>
 </file>
@@ -1092,87 +1092,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1183,6 +1102,87 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1519,7 +1519,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -1535,7 +1535,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -1551,7 +1551,7 @@
         <v>100</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1606,17 +1606,17 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="78" t="s">
+      <c r="A2" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" s="52" t="s">
         <v>104</v>
       </c>
-      <c r="B2" s="79" t="s">
+      <c r="C2" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="80" t="s">
-        <v>106</v>
-      </c>
       <c r="D2" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E2" s="47">
         <v>25227</v>
@@ -1632,17 +1632,17 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B3" s="79" t="s">
+      <c r="A3" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="52" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>107</v>
-      </c>
-      <c r="C3" s="80" t="s">
-        <v>106</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>108</v>
       </c>
       <c r="E3" s="47">
         <v>10813</v>
@@ -1658,17 +1658,17 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="79" t="s">
+      <c r="A4" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" s="52" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="C4" s="80" t="s">
-        <v>106</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>110</v>
       </c>
       <c r="E4" s="47">
         <v>42579</v>
@@ -1684,17 +1684,17 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" s="79" t="s">
+      <c r="A5" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="52" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>111</v>
-      </c>
-      <c r="C5" s="80" t="s">
-        <v>106</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>112</v>
       </c>
       <c r="E5" s="47">
         <v>77422</v>
@@ -1710,17 +1710,17 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B6" s="79" t="s">
+      <c r="A6" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="52" t="s">
+        <v>112</v>
+      </c>
+      <c r="C6" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="C6" s="80" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>114</v>
       </c>
       <c r="E6" s="47">
         <v>29805</v>
@@ -1736,17 +1736,17 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B7" s="79" t="s">
+      <c r="A7" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="52" t="s">
+        <v>114</v>
+      </c>
+      <c r="C7" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="C7" s="80" t="s">
-        <v>106</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>116</v>
       </c>
       <c r="E7" s="47">
         <v>9546</v>
@@ -1781,53 +1781,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="49" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="58" t="s">
+      <c r="C1" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="53" t="s">
+      <c r="E1" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="F1" s="53" t="s">
+      <c r="F1" s="56" t="s">
         <v>92</v>
       </c>
-      <c r="G1" s="53" t="s">
+      <c r="G1" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="55" t="s">
+      <c r="H1" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="51" t="s">
+      <c r="I1" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="51"/>
-      <c r="K1" s="51"/>
-      <c r="L1" s="51"/>
-      <c r="M1" s="51"/>
-      <c r="N1" s="51" t="s">
+      <c r="J1" s="54"/>
+      <c r="K1" s="54"/>
+      <c r="L1" s="54"/>
+      <c r="M1" s="54"/>
+      <c r="N1" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="51" t="s">
+      <c r="O1" s="54" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="57"/>
-      <c r="B2" s="57"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="56"/>
+      <c r="A2" s="60"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="59"/>
       <c r="I2" s="43">
         <v>2018</v>
       </c>
@@ -1843,21 +1843,21 @@
       <c r="M2" s="43">
         <v>2022</v>
       </c>
-      <c r="N2" s="52"/>
-      <c r="O2" s="52"/>
+      <c r="N2" s="55"/>
+      <c r="O2" s="55"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="52" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="79" t="s">
+      <c r="C3" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="C3" s="80" t="s">
-        <v>106</v>
-      </c>
       <c r="D3" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E3" s="47"/>
       <c r="F3" s="47"/>
@@ -1890,17 +1890,17 @@
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="79" t="s">
+      <c r="A4" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" s="52" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>107</v>
-      </c>
-      <c r="C4" s="80" t="s">
-        <v>106</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>108</v>
       </c>
       <c r="E4" s="47"/>
       <c r="F4" s="47"/>
@@ -1933,17 +1933,17 @@
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" s="79" t="s">
+      <c r="A5" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="52" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="C5" s="80" t="s">
-        <v>106</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>110</v>
       </c>
       <c r="E5" s="47"/>
       <c r="F5" s="47"/>
@@ -1976,17 +1976,17 @@
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B6" s="79" t="s">
+      <c r="A6" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="52" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>111</v>
-      </c>
-      <c r="C6" s="80" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>112</v>
       </c>
       <c r="E6" s="47"/>
       <c r="F6" s="47"/>
@@ -2019,17 +2019,17 @@
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B7" s="79" t="s">
+      <c r="A7" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="52" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="C7" s="80" t="s">
-        <v>106</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>114</v>
       </c>
       <c r="E7" s="47"/>
       <c r="F7" s="47"/>
@@ -2062,17 +2062,17 @@
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B8" s="79" t="s">
+      <c r="A8" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="52" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" s="53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="C8" s="80" t="s">
-        <v>106</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>116</v>
       </c>
       <c r="E8" s="47"/>
       <c r="F8" s="47"/>
@@ -2146,53 +2146,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="58" t="s">
+      <c r="C1" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="53" t="s">
+      <c r="E1" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="F1" s="53" t="s">
+      <c r="F1" s="56" t="s">
         <v>92</v>
       </c>
-      <c r="G1" s="53" t="s">
+      <c r="G1" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="55" t="s">
+      <c r="H1" s="58" t="s">
         <v>44</v>
       </c>
       <c r="I1" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="59" t="s">
+      <c r="J1" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
       <c r="O1" s="44" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="91" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="57"/>
-      <c r="B2" s="57"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="56"/>
+      <c r="A2" s="60"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="59"/>
       <c r="I2" s="44" t="s">
         <v>15</v>
       </c>
@@ -2216,17 +2216,17 @@
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="52" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="79" t="s">
+      <c r="C3" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>106</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E3" s="47"/>
       <c r="F3" s="47"/>
@@ -2259,17 +2259,17 @@
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="79" t="s">
+      <c r="A4" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" s="52" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="E4" s="47"/>
       <c r="F4" s="47"/>
@@ -2292,17 +2292,17 @@
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" s="79" t="s">
+      <c r="A5" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="52" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="E5" s="47"/>
       <c r="F5" s="47"/>
@@ -2325,17 +2325,17 @@
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B6" s="79" t="s">
+      <c r="A6" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="52" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="E6" s="47"/>
       <c r="F6" s="47"/>
@@ -2368,17 +2368,17 @@
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B7" s="79" t="s">
+      <c r="A7" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="52" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="E7" s="47"/>
       <c r="F7" s="47"/>
@@ -2401,17 +2401,17 @@
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B8" s="79" t="s">
+      <c r="A8" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="52" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="E8" s="47"/>
       <c r="F8" s="47"/>
@@ -2466,28 +2466,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="48" x14ac:dyDescent="0.2">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="58" t="s">
+      <c r="C1" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="53" t="s">
+      <c r="E1" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="F1" s="53" t="s">
+      <c r="F1" s="56" t="s">
         <v>92</v>
       </c>
-      <c r="G1" s="53" t="s">
+      <c r="G1" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="55" t="s">
+      <c r="H1" s="58" t="s">
         <v>44</v>
       </c>
       <c r="I1" s="45" t="s">
@@ -2498,14 +2498,14 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="48" x14ac:dyDescent="0.2">
-      <c r="A2" s="57"/>
-      <c r="B2" s="57"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="56"/>
+      <c r="A2" s="60"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="59"/>
       <c r="I2" s="45" t="s">
         <v>25</v>
       </c>
@@ -2514,17 +2514,17 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="52" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="79" t="s">
+      <c r="C3" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>106</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E3" s="47"/>
       <c r="F3" s="47"/>
@@ -2542,17 +2542,17 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="79" t="s">
+      <c r="A4" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" s="52" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="E4" s="47"/>
       <c r="F4" s="47"/>
@@ -2570,17 +2570,17 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" s="79" t="s">
+      <c r="A5" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="52" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="E5" s="47"/>
       <c r="F5" s="47"/>
@@ -2598,17 +2598,17 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B6" s="79" t="s">
+      <c r="A6" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="52" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="E6" s="47"/>
       <c r="F6" s="47"/>
@@ -2626,17 +2626,17 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B7" s="79" t="s">
+      <c r="A7" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="52" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="E7" s="47"/>
       <c r="F7" s="47"/>
@@ -2654,17 +2654,17 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B8" s="79" t="s">
+      <c r="A8" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="52" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="E8" s="47"/>
       <c r="F8" s="47"/>
@@ -2710,48 +2710,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="58" t="s">
+      <c r="C1" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="53" t="s">
+      <c r="E1" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="F1" s="53" t="s">
+      <c r="F1" s="56" t="s">
         <v>92</v>
       </c>
-      <c r="G1" s="53" t="s">
+      <c r="G1" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="55" t="s">
+      <c r="H1" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="61" t="s">
+      <c r="I1" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+      <c r="N1" s="65"/>
     </row>
     <row r="2" spans="1:14" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="57"/>
-      <c r="B2" s="57"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="56"/>
+      <c r="A2" s="60"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="59"/>
       <c r="I2" s="46" t="s">
         <v>93</v>
       </c>
@@ -2772,17 +2772,17 @@
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="52" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="79" t="s">
+      <c r="C3" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>106</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E3" s="47"/>
       <c r="F3" s="47"/>
@@ -2812,17 +2812,17 @@
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="79" t="s">
+      <c r="A4" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" s="52" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="E4" s="47"/>
       <c r="F4" s="47"/>
@@ -2852,17 +2852,17 @@
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A5" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" s="79" t="s">
+      <c r="A5" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="52" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="E5" s="47"/>
       <c r="F5" s="47"/>
@@ -2892,17 +2892,17 @@
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A6" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B6" s="79" t="s">
+      <c r="A6" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="52" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="E6" s="47"/>
       <c r="F6" s="47"/>
@@ -2932,17 +2932,17 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A7" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B7" s="79" t="s">
+      <c r="A7" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="52" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="E7" s="47"/>
       <c r="F7" s="47"/>
@@ -2972,17 +2972,17 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A8" s="78" t="s">
-        <v>104</v>
-      </c>
-      <c r="B8" s="79" t="s">
+      <c r="A8" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="52" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="E8" s="47"/>
       <c r="F8" s="47"/>
@@ -3062,7 +3062,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="74" t="s">
         <v>81</v>
       </c>
       <c r="B2" s="37" t="s">
@@ -3073,7 +3073,7 @@
       <c r="E2" s="22"/>
     </row>
     <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="72"/>
+      <c r="A3" s="75"/>
       <c r="B3" s="38" t="s">
         <v>7</v>
       </c>
@@ -3082,7 +3082,7 @@
       <c r="E3" s="24"/>
     </row>
     <row r="4" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A4" s="72"/>
+      <c r="A4" s="75"/>
       <c r="B4" s="31" t="s">
         <v>8</v>
       </c>
@@ -3095,7 +3095,7 @@
       <c r="E4" s="24"/>
     </row>
     <row r="5" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="72"/>
+      <c r="A5" s="75"/>
       <c r="B5" s="38" t="s">
         <v>9</v>
       </c>
@@ -3108,7 +3108,7 @@
       <c r="E5" s="24"/>
     </row>
     <row r="6" spans="1:5" ht="33" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="73"/>
+      <c r="A6" s="76"/>
       <c r="B6" s="39" t="s">
         <v>94</v>
       </c>
@@ -3121,7 +3121,7 @@
       <c r="E6" s="50"/>
     </row>
     <row r="7" spans="1:5" ht="35" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="73"/>
+      <c r="A7" s="76"/>
       <c r="B7" s="39" t="s">
         <v>10</v>
       </c>
@@ -3134,7 +3134,7 @@
       <c r="E7" s="50"/>
     </row>
     <row r="8" spans="1:5" ht="35" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="74"/>
+      <c r="A8" s="77"/>
       <c r="B8" s="39" t="s">
         <v>10</v>
       </c>
@@ -3147,7 +3147,7 @@
       <c r="E8" s="25"/>
     </row>
     <row r="9" spans="1:5" ht="85" x14ac:dyDescent="0.2">
-      <c r="A9" s="75" t="s">
+      <c r="A9" s="78" t="s">
         <v>82</v>
       </c>
       <c r="B9" s="10" t="s">
@@ -3164,7 +3164,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A10" s="76"/>
+      <c r="A10" s="79"/>
       <c r="B10" s="16" t="s">
         <v>48</v>
       </c>
@@ -3177,7 +3177,7 @@
       <c r="E10" s="15"/>
     </row>
     <row r="11" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A11" s="76"/>
+      <c r="A11" s="79"/>
       <c r="B11" s="16" t="s">
         <v>50</v>
       </c>
@@ -3192,7 +3192,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="97" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="77"/>
+      <c r="A12" s="80"/>
       <c r="B12" s="19" t="s">
         <v>13</v>
       </c>
@@ -3207,7 +3207,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="64" x14ac:dyDescent="0.2">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="66" t="s">
         <v>56</v>
       </c>
       <c r="B13" s="16" t="s">
@@ -3224,7 +3224,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="96" x14ac:dyDescent="0.2">
-      <c r="A14" s="64"/>
+      <c r="A14" s="67"/>
       <c r="B14" s="16" t="s">
         <v>59</v>
       </c>
@@ -3239,7 +3239,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="96" x14ac:dyDescent="0.2">
-      <c r="A15" s="64"/>
+      <c r="A15" s="67"/>
       <c r="B15" s="16" t="s">
         <v>18</v>
       </c>
@@ -3254,7 +3254,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="96" x14ac:dyDescent="0.2">
-      <c r="A16" s="64"/>
+      <c r="A16" s="67"/>
       <c r="B16" s="16" t="s">
         <v>19</v>
       </c>
@@ -3269,7 +3269,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="96" x14ac:dyDescent="0.2">
-      <c r="A17" s="64"/>
+      <c r="A17" s="67"/>
       <c r="B17" s="16" t="s">
         <v>64</v>
       </c>
@@ -3284,7 +3284,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="96" x14ac:dyDescent="0.2">
-      <c r="A18" s="64"/>
+      <c r="A18" s="67"/>
       <c r="B18" s="16" t="s">
         <v>21</v>
       </c>
@@ -3299,7 +3299,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="129" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="65"/>
+      <c r="A19" s="68"/>
       <c r="B19" s="32" t="s">
         <v>23</v>
       </c>
@@ -3314,7 +3314,7 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="160" x14ac:dyDescent="0.2">
-      <c r="A20" s="66" t="s">
+      <c r="A20" s="69" t="s">
         <v>69</v>
       </c>
       <c r="B20" s="34" t="s">
@@ -3330,8 +3330,8 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="113" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="67"/>
+    <row r="21" spans="1:5" ht="97" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="70"/>
       <c r="B21" s="29" t="s">
         <v>27</v>
       </c>
@@ -3346,7 +3346,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A22" s="68" t="s">
+      <c r="A22" s="71" t="s">
         <v>83</v>
       </c>
       <c r="B22" s="34" t="s">
@@ -3361,7 +3361,7 @@
       <c r="E22" s="13"/>
     </row>
     <row r="23" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A23" s="69"/>
+      <c r="A23" s="72"/>
       <c r="B23" s="35" t="s">
         <v>74</v>
       </c>
@@ -3374,7 +3374,7 @@
       <c r="E23" s="15"/>
     </row>
     <row r="24" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A24" s="69"/>
+      <c r="A24" s="72"/>
       <c r="B24" s="35" t="s">
         <v>31</v>
       </c>
@@ -3387,7 +3387,7 @@
       <c r="E24" s="15"/>
     </row>
     <row r="25" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A25" s="69"/>
+      <c r="A25" s="72"/>
       <c r="B25" s="35" t="s">
         <v>32</v>
       </c>
@@ -3399,8 +3399,8 @@
       </c>
       <c r="E25" s="15"/>
     </row>
-    <row r="26" spans="1:5" ht="49" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="70"/>
+    <row r="26" spans="1:5" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="73"/>
       <c r="B26" s="29" t="s">
         <v>78</v>
       </c>

</xml_diff>